<commit_message>
implement req prompt v2
</commit_message>
<xml_diff>
--- a/resource/groundTruths/requirement/CF_M05_ground_truth_requirement.xlsx
+++ b/resource/groundTruths/requirement/CF_M05_ground_truth_requirement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oguzarslan/Desktop/upc/semester-4/Thesis/MappingGenerator/resource/groundTruths/requirement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6234FAA-E1E0-A546-A443-C46521E39213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8320D5BB-EC30-9C4C-9BA5-BDFA7B47F9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14800" yWindow="900" windowWidth="14440" windowHeight="16580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14800" yWindow="900" windowWidth="14440" windowHeight="16580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="104">
   <si>
     <t>Document ID</t>
   </si>
@@ -335,6 +335,9 @@
   </si>
   <si>
     <t>*CF_M05_C18</t>
+  </si>
+  <si>
+    <t>No user can access data from other customers.</t>
   </si>
 </sst>
 </file>
@@ -1210,6 +1213,9 @@
       <c r="B26" t="s">
         <v>83</v>
       </c>
+      <c r="C26" t="s">
+        <v>103</v>
+      </c>
       <c r="D26" t="s">
         <v>31</v>
       </c>

</xml_diff>